<commit_message>
Upload new-aia-mdu-addresses/New AIA MDU Addresses.xlsx via form
</commit_message>
<xml_diff>
--- a/inbox/new-aia-mdu-addresses/New AIA MDU Addresses.xlsx
+++ b/inbox/new-aia-mdu-addresses/New AIA MDU Addresses.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="All Addresses" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Copy of All Addresses" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,14 +11,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="43">
   <si>
     <t>Full Address</t>
   </si>
   <si>
+    <t>State</t>
+  </si>
+  <si>
     <t>23733 N SCOTTSDALE RD, SCOTTSDALE 85255</t>
   </si>
   <si>
+    <t>AZ</t>
+  </si>
+  <si>
     <t>42015 N VENTURE DR, PHOENIX 85086</t>
   </si>
   <si>
@@ -67,6 +73,9 @@
     <t>3602 N NARROWS DR, TACOMA 98407</t>
   </si>
   <si>
+    <t>WA</t>
+  </si>
+  <si>
     <t>1201 HANCOCK ST, PORT TOWNSEND 98368</t>
   </si>
   <si>
@@ -91,28 +100,43 @@
     <t>340 NE CREST ST, SUBLIMITY 97385</t>
   </si>
   <si>
+    <t>OR</t>
+  </si>
+  <si>
     <t>21599 DOLORES WAY NE, AURORA 97002</t>
   </si>
   <si>
     <t>1565 N UNIVERSITY AVE, PROVO 84604</t>
   </si>
   <si>
+    <t>UT</t>
+  </si>
+  <si>
     <t>3375 W MOUNT ELLEN WAY, SALT LAKE CITY 84129</t>
   </si>
   <si>
     <t>1150 VINYARD RD, VINTON 24179</t>
   </si>
   <si>
+    <t>VA</t>
+  </si>
+  <si>
     <t>209 OLD GRAVES MILL RD, LYNCHBURG 24502</t>
   </si>
   <si>
     <t>221 SCOTT ST, WAUSAU 54403</t>
   </si>
   <si>
+    <t>WI</t>
+  </si>
+  <si>
     <t>711 E 1ST ST, MERRILL 54452</t>
   </si>
   <si>
     <t>1700 W PLUM ST, FORT COLLINS 80521</t>
+  </si>
+  <si>
+    <t>CO</t>
   </si>
   <si>
     <t>310 N MASON ST, FORT COLLINS 80524</t>
@@ -155,13 +179,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -380,182 +405,288 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="46.0"/>
+    <col customWidth="1" min="1" max="1" width="42.5"/>
+    <col customWidth="1" min="2" max="2" width="5.13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
+      <c r="A3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>5</v>
+      <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>6</v>
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>7</v>
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>8</v>
+      <c r="A9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
+      <c r="A10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>10</v>
+      <c r="A11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>11</v>
+      <c r="A12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>12</v>
+      <c r="A13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
+      <c r="A14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>14</v>
+      <c r="A15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
-        <v>15</v>
+      <c r="A16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="s">
-        <v>16</v>
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="s">
-        <v>17</v>
+      <c r="A18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="s">
-        <v>18</v>
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="s">
-        <v>19</v>
+      <c r="A20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="s">
-        <v>21</v>
+      <c r="A22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="s">
-        <v>22</v>
+      <c r="A23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="s">
-        <v>23</v>
+      <c r="A24" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="s">
-        <v>24</v>
+      <c r="A25" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="s">
-        <v>25</v>
+      <c r="A26" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="s">
-        <v>26</v>
+      <c r="A27" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="s">
-        <v>27</v>
+      <c r="A28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="s">
-        <v>28</v>
+      <c r="A29" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="s">
-        <v>29</v>
+      <c r="A30" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="s">
-        <v>30</v>
+      <c r="A31" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="s">
-        <v>31</v>
+      <c r="A32" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="s">
-        <v>32</v>
+      <c r="A33" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="s">
-        <v>33</v>
+      <c r="A34" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="s">
-        <v>34</v>
+      <c r="A35" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>